<commit_message>
Created the desrialized data in the form of [{"Name":"Neid","VendorAddress":"..."}] using data table.
</commit_message>
<xml_diff>
--- a/AP.InvoicePerformer/Data/Exports/invoice-3-2_1-1.xlsx
+++ b/AP.InvoicePerformer/Data/Exports/invoice-3-2_1-1.xlsx
@@ -109,13 +109,13 @@
     <x:t>12580</x:t>
   </x:si>
   <x:si>
+    <x:t>143380</x:t>
+  </x:si>
+  <x:si>
+    <x:t>table</x:t>
+  </x:si>
+  <x:si>
     <x:t>125800</x:t>
-  </x:si>
-  <x:si>
-    <x:t>143380</x:t>
-  </x:si>
-  <x:si>
-    <x:t>table</x:t>
   </x:si>
   <x:si>
     <x:t>Key,Value
@@ -142,6 +142,9 @@
 "Zip Postal Code","26655"</x:t>
   </x:si>
   <x:si>
+    <x:t>125800.00</x:t>
+  </x:si>
+  <x:si>
     <x:t>Line Number</x:t>
   </x:si>
   <x:si>
@@ -169,28 +172,43 @@
     <x:t>459-83-1839</x:t>
   </x:si>
   <x:si>
+    <x:t>13700</x:t>
+  </x:si>
+  <x:si>
     <x:t>Ford/Mustang Country of origin: Portugal Color: Black</x:t>
   </x:si>
   <x:si>
     <x:t>678-29-5664</x:t>
   </x:si>
   <x:si>
+    <x:t>19600</x:t>
+  </x:si>
+  <x:si>
     <x:t>Aston Martin/V8 Vantage Country of origin: Portugal Color: Black</x:t>
   </x:si>
   <x:si>
     <x:t>815-12-9380</x:t>
   </x:si>
   <x:si>
+    <x:t>22600</x:t>
+  </x:si>
+  <x:si>
     <x:t>Lamborghini/Gallardo Country of origin: France Color: Silver</x:t>
   </x:si>
   <x:si>
     <x:t>224-17-7360</x:t>
   </x:si>
   <x:si>
+    <x:t>40500</x:t>
+  </x:si>
+  <x:si>
     <x:t>Mercedes-Benz/G-Class Country of origin: Germany Color: Blue</x:t>
   </x:si>
   <x:si>
-    <x:t>0</x:t>
+    <x:t>542-58-1039</x:t>
+  </x:si>
+  <x:si>
+    <x:t>2940 0</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -641,13 +659,13 @@
       <x:c r="O2" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="P2" s="0" t="s">
+      <x:c r="Q2" s="0" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="Q2" s="0" t="s">
+      <x:c r="S2" s="0" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="S2" s="0" t="s">
+      <x:c r="T2" s="0" t="s">
         <x:v>32</x:v>
       </x:c>
     </x:row>
@@ -761,14 +779,14 @@
       <x:c r="O2" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
-      <x:c r="P2" s="0" t="s">
+      <x:c r="Q2" s="0" t="s">
         <x:v>30</x:v>
       </x:c>
-      <x:c r="Q2" s="0" t="s">
+      <x:c r="S2" s="0" t="s">
         <x:v>31</x:v>
       </x:c>
-      <x:c r="S2" s="0" t="s">
-        <x:v>32</x:v>
+      <x:c r="T2" s="0" t="s">
+        <x:v>36</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -790,65 +808,80 @@
   <x:sheetData>
     <x:row r="1" spans="1:7">
       <x:c r="A1" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7">
       <x:c r="B2" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G2" s="0" t="s">
         <x:v>44</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
       <x:c r="B3" s="0" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
       <x:c r="B4" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="G4" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="B5" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="G5" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
       <x:c r="B6" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F6" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>58</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -870,65 +903,80 @@
   <x:sheetData>
     <x:row r="1" spans="1:7">
       <x:c r="A1" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>37</x:v>
       </x:c>
       <x:c r="B1" s="0" t="s">
-        <x:v>37</x:v>
+        <x:v>38</x:v>
       </x:c>
       <x:c r="C1" s="0" t="s">
-        <x:v>38</x:v>
+        <x:v>39</x:v>
       </x:c>
       <x:c r="D1" s="0" t="s">
-        <x:v>39</x:v>
+        <x:v>40</x:v>
       </x:c>
       <x:c r="E1" s="0" t="s">
-        <x:v>40</x:v>
+        <x:v>41</x:v>
       </x:c>
       <x:c r="F1" s="0" t="s">
-        <x:v>41</x:v>
+        <x:v>42</x:v>
       </x:c>
       <x:c r="G1" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7">
       <x:c r="B2" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="G2" s="0" t="s">
         <x:v>44</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>45</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
       <x:c r="B3" s="0" t="s">
-        <x:v>45</x:v>
-      </x:c>
-      <x:c r="G3" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="C3" s="0" t="s">
+        <x:v>48</x:v>
+      </x:c>
+      <x:c r="E3" s="0" t="s">
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
       <x:c r="B4" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="G4" s="0" t="s">
-        <x:v>48</x:v>
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="C4" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="E4" s="0" t="s">
+        <x:v>52</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="B5" s="0" t="s">
-        <x:v>49</x:v>
-      </x:c>
-      <x:c r="G5" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="C5" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="E5" s="0" t="s">
+        <x:v>55</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
       <x:c r="B6" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="F6" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>58</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Corrected the appURL and made some changes in performer
</commit_message>
<xml_diff>
--- a/AP.InvoicePerformer/Data/Exports/invoice-3-2_1-1.xlsx
+++ b/AP.InvoicePerformer/Data/Exports/invoice-3-2_1-1.xlsx
@@ -109,13 +109,13 @@
     <x:t>12580</x:t>
   </x:si>
   <x:si>
+    <x:t>125800</x:t>
+  </x:si>
+  <x:si>
     <x:t>143380</x:t>
   </x:si>
   <x:si>
     <x:t>table</x:t>
-  </x:si>
-  <x:si>
-    <x:t>125800</x:t>
   </x:si>
   <x:si>
     <x:t>Key,Value
@@ -142,9 +142,6 @@
 "Zip Postal Code","26655"</x:t>
   </x:si>
   <x:si>
-    <x:t>125800.00</x:t>
-  </x:si>
-  <x:si>
     <x:t>Line Number</x:t>
   </x:si>
   <x:si>
@@ -166,7 +163,7 @@
     <x:t>Part Number</x:t>
   </x:si>
   <x:si>
-    <x:t>Spyker/C8 Spyder Wide Body Country of origin: Germany Color: Silver</x:t>
+    <x:t>Spyker/C8 Spyder Wide Body</x:t>
   </x:si>
   <x:si>
     <x:t>459-83-1839</x:t>
@@ -175,7 +172,10 @@
     <x:t>13700</x:t>
   </x:si>
   <x:si>
-    <x:t>Ford/Mustang Country of origin: Portugal Color: Black</x:t>
+    <x:t>Country of origin: Germany Color: Silver</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Ford/Mustang</x:t>
   </x:si>
   <x:si>
     <x:t>678-29-5664</x:t>
@@ -184,7 +184,10 @@
     <x:t>19600</x:t>
   </x:si>
   <x:si>
-    <x:t>Aston Martin/V8 Vantage Country of origin: Portugal Color: Black</x:t>
+    <x:t>Country of origin: Portugal Color: Black</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Aston Martin/V8 Vantage</x:t>
   </x:si>
   <x:si>
     <x:t>815-12-9380</x:t>
@@ -193,7 +196,7 @@
     <x:t>22600</x:t>
   </x:si>
   <x:si>
-    <x:t>Lamborghini/Gallardo Country of origin: France Color: Silver</x:t>
+    <x:t>Lamborghini/Gallardo</x:t>
   </x:si>
   <x:si>
     <x:t>224-17-7360</x:t>
@@ -202,13 +205,19 @@
     <x:t>40500</x:t>
   </x:si>
   <x:si>
-    <x:t>Mercedes-Benz/G-Class Country of origin: Germany Color: Blue</x:t>
+    <x:t>Country of origin: France Color: Silver</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Mercedes-Benz/G-Class</x:t>
   </x:si>
   <x:si>
     <x:t>542-58-1039</x:t>
   </x:si>
   <x:si>
     <x:t>2940 0</x:t>
+  </x:si>
+  <x:si>
+    <x:t>Country of origin: Germany Color: Blue</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -659,13 +668,13 @@
       <x:c r="O2" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
+      <x:c r="P2" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="Q2" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="S2" s="0" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="T2" s="0" t="s">
         <x:v>32</x:v>
       </x:c>
     </x:row>
@@ -779,14 +788,14 @@
       <x:c r="O2" s="0" t="s">
         <x:v>29</x:v>
       </x:c>
+      <x:c r="P2" s="0" t="s">
+        <x:v>30</x:v>
+      </x:c>
       <x:c r="Q2" s="0" t="s">
-        <x:v>30</x:v>
+        <x:v>31</x:v>
       </x:c>
       <x:c r="S2" s="0" t="s">
-        <x:v>31</x:v>
-      </x:c>
-      <x:c r="T2" s="0" t="s">
-        <x:v>36</x:v>
+        <x:v>32</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -808,80 +817,105 @@
   <x:sheetData>
     <x:row r="1" spans="1:7">
       <x:c r="A1" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
+      <x:c r="C1" s="0" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="C1" s="0" t="s">
+      <x:c r="D1" s="0" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="D1" s="0" t="s">
+      <x:c r="E1" s="0" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="E1" s="0" t="s">
+      <x:c r="F1" s="0" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="F1" s="0" t="s">
+      <x:c r="G1" s="0" t="s">
         <x:v>42</x:v>
-      </x:c>
-      <x:c r="G1" s="0" t="s">
-        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7">
       <x:c r="B2" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="C2" s="0" t="s">
+      <x:c r="E2" s="0" t="s">
         <x:v>45</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
-        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
       <x:c r="B3" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
       <x:c r="B4" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="B5" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
       <x:c r="B6" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:7">
+      <x:c r="B7" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:7">
+      <x:c r="B8" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="C6" s="0" t="s">
+    </x:row>
+    <x:row r="9" spans="1:7">
+      <x:c r="B9" s="0" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="E6" s="0" t="s">
+    </x:row>
+    <x:row r="10" spans="1:7">
+      <x:c r="B10" s="0" t="s">
         <x:v>58</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:7">
+      <x:c r="B11" s="0" t="s">
+        <x:v>61</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -903,80 +937,105 @@
   <x:sheetData>
     <x:row r="1" spans="1:7">
       <x:c r="A1" s="0" t="s">
+        <x:v>36</x:v>
+      </x:c>
+      <x:c r="B1" s="0" t="s">
         <x:v>37</x:v>
       </x:c>
-      <x:c r="B1" s="0" t="s">
+      <x:c r="C1" s="0" t="s">
         <x:v>38</x:v>
       </x:c>
-      <x:c r="C1" s="0" t="s">
+      <x:c r="D1" s="0" t="s">
         <x:v>39</x:v>
       </x:c>
-      <x:c r="D1" s="0" t="s">
+      <x:c r="E1" s="0" t="s">
         <x:v>40</x:v>
       </x:c>
-      <x:c r="E1" s="0" t="s">
+      <x:c r="F1" s="0" t="s">
         <x:v>41</x:v>
       </x:c>
-      <x:c r="F1" s="0" t="s">
+      <x:c r="G1" s="0" t="s">
         <x:v>42</x:v>
-      </x:c>
-      <x:c r="G1" s="0" t="s">
-        <x:v>43</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7">
       <x:c r="B2" s="0" t="s">
+        <x:v>43</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
         <x:v>44</x:v>
       </x:c>
-      <x:c r="C2" s="0" t="s">
+      <x:c r="E2" s="0" t="s">
         <x:v>45</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
-        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:7">
       <x:c r="B3" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="C3" s="0" t="s">
-        <x:v>48</x:v>
-      </x:c>
-      <x:c r="E3" s="0" t="s">
-        <x:v>49</x:v>
+        <x:v>46</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
       <x:c r="B4" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>51</x:v>
+        <x:v>48</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
-        <x:v>52</x:v>
+        <x:v>49</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:7">
       <x:c r="B5" s="0" t="s">
-        <x:v>53</x:v>
-      </x:c>
-      <x:c r="C5" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E5" s="0" t="s">
-        <x:v>55</x:v>
+        <x:v>50</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
       <x:c r="B6" s="0" t="s">
+        <x:v>51</x:v>
+      </x:c>
+      <x:c r="C6" s="0" t="s">
+        <x:v>52</x:v>
+      </x:c>
+      <x:c r="E6" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7" spans="1:7">
+      <x:c r="B7" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" spans="1:7">
+      <x:c r="B8" s="0" t="s">
+        <x:v>54</x:v>
+      </x:c>
+      <x:c r="C8" s="0" t="s">
+        <x:v>55</x:v>
+      </x:c>
+      <x:c r="E8" s="0" t="s">
         <x:v>56</x:v>
       </x:c>
-      <x:c r="C6" s="0" t="s">
+    </x:row>
+    <x:row r="9" spans="1:7">
+      <x:c r="B9" s="0" t="s">
         <x:v>57</x:v>
       </x:c>
-      <x:c r="E6" s="0" t="s">
+    </x:row>
+    <x:row r="10" spans="1:7">
+      <x:c r="B10" s="0" t="s">
         <x:v>58</x:v>
+      </x:c>
+      <x:c r="C10" s="0" t="s">
+        <x:v>59</x:v>
+      </x:c>
+      <x:c r="E10" s="0" t="s">
+        <x:v>60</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" spans="1:7">
+      <x:c r="B11" s="0" t="s">
+        <x:v>61</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Added invoke code activity for passing the datatable to the app instead of passing the json string
</commit_message>
<xml_diff>
--- a/AP.InvoicePerformer/Data/Exports/invoice-3-2_1-1.xlsx
+++ b/AP.InvoicePerformer/Data/Exports/invoice-3-2_1-1.xlsx
@@ -150,37 +150,40 @@
     <x:t>Part Number</x:t>
   </x:si>
   <x:si>
+    <x:t>13700</x:t>
+  </x:si>
+  <x:si>
     <x:t>Spyker/C8 Spyder Wide Body</x:t>
   </x:si>
   <x:si>
     <x:t>459-83-1839</x:t>
   </x:si>
   <x:si>
-    <x:t>13700</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: Germany Color: Silver</x:t>
   </x:si>
   <x:si>
+    <x:t>19600</x:t>
+  </x:si>
+  <x:si>
     <x:t>Ford/Mustang</x:t>
   </x:si>
   <x:si>
     <x:t>678-29-5664</x:t>
   </x:si>
   <x:si>
-    <x:t>19600</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: Portugal Color: Black</x:t>
   </x:si>
   <x:si>
+    <x:t>22600</x:t>
+  </x:si>
+  <x:si>
     <x:t>Aston Martin/V8 Vantage</x:t>
   </x:si>
   <x:si>
     <x:t>815-12-9380</x:t>
   </x:si>
   <x:si>
-    <x:t>22600</x:t>
+    <x:t>40500</x:t>
   </x:si>
   <x:si>
     <x:t>Lamborghini/Gallardo</x:t>
@@ -189,19 +192,16 @@
     <x:t>224-17-7360</x:t>
   </x:si>
   <x:si>
-    <x:t>40500</x:t>
-  </x:si>
-  <x:si>
     <x:t>Country of origin: France Color: Silver</x:t>
   </x:si>
   <x:si>
+    <x:t>2940 0</x:t>
+  </x:si>
+  <x:si>
     <x:t>Mercedes-Benz/G-Class</x:t>
   </x:si>
   <x:si>
     <x:t>542-58-1039</x:t>
-  </x:si>
-  <x:si>
-    <x:t>2940 0</x:t>
   </x:si>
   <x:si>
     <x:t>Country of origin: Germany Color: Blue</x:t>
@@ -664,9 +664,6 @@
       <x:c r="N2" s="0" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="S2" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -787,9 +784,6 @@
       <x:c r="N2" s="0" t="s">
         <x:v>32</x:v>
       </x:c>
-      <x:c r="S2" s="0" t="s">
-        <x:v>30</x:v>
-      </x:c>
     </x:row>
   </x:sheetData>
   <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
@@ -832,13 +826,13 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7">
+      <x:c r="A2" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
         <x:v>44</x:v>
       </x:c>
     </x:row>
@@ -848,13 +842,13 @@
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
+      <x:c r="A4" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
         <x:v>48</x:v>
       </x:c>
     </x:row>
@@ -864,13 +858,13 @@
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
+      <x:c r="A6" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
         <x:v>52</x:v>
       </x:c>
     </x:row>
@@ -880,13 +874,13 @@
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7">
+      <x:c r="A8" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
         <x:v>55</x:v>
       </x:c>
     </x:row>
@@ -896,13 +890,13 @@
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7">
+      <x:c r="A10" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="E10" s="0" t="s">
         <x:v>59</x:v>
       </x:c>
     </x:row>
@@ -952,13 +946,13 @@
       </x:c>
     </x:row>
     <x:row r="2" spans="1:7">
+      <x:c r="A2" s="0" t="s">
+        <x:v>42</x:v>
+      </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>42</x:v>
+        <x:v>43</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>43</x:v>
-      </x:c>
-      <x:c r="E2" s="0" t="s">
         <x:v>44</x:v>
       </x:c>
     </x:row>
@@ -968,13 +962,13 @@
       </x:c>
     </x:row>
     <x:row r="4" spans="1:7">
+      <x:c r="A4" s="0" t="s">
+        <x:v>46</x:v>
+      </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>46</x:v>
+        <x:v>47</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>47</x:v>
-      </x:c>
-      <x:c r="E4" s="0" t="s">
         <x:v>48</x:v>
       </x:c>
     </x:row>
@@ -984,13 +978,13 @@
       </x:c>
     </x:row>
     <x:row r="6" spans="1:7">
+      <x:c r="A6" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>50</x:v>
+        <x:v>51</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>51</x:v>
-      </x:c>
-      <x:c r="E6" s="0" t="s">
         <x:v>52</x:v>
       </x:c>
     </x:row>
@@ -1000,13 +994,13 @@
       </x:c>
     </x:row>
     <x:row r="8" spans="1:7">
+      <x:c r="A8" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>53</x:v>
+        <x:v>54</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>54</x:v>
-      </x:c>
-      <x:c r="E8" s="0" t="s">
         <x:v>55</x:v>
       </x:c>
     </x:row>
@@ -1016,13 +1010,13 @@
       </x:c>
     </x:row>
     <x:row r="10" spans="1:7">
+      <x:c r="A10" s="0" t="s">
+        <x:v>57</x:v>
+      </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>57</x:v>
+        <x:v>58</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>58</x:v>
-      </x:c>
-      <x:c r="E10" s="0" t="s">
         <x:v>59</x:v>
       </x:c>
     </x:row>

</xml_diff>